<commit_message>
added english and set as default
</commit_message>
<xml_diff>
--- a/data/spellforce_soundtrack_data.xlsx
+++ b/data/spellforce_soundtrack_data.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">locations!$A$1:$F$224</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">maps!$A$1:$G$49</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">maps!$A$1:$H$49</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">songs!$A$1:$C$71</definedName>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">tracks!$A$1:$C$198</definedName>
   </definedNames>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="913" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="962" uniqueCount="338">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -484,6 +484,9 @@
     <t xml:space="preserve">mapSort</t>
   </si>
   <si>
+    <t xml:space="preserve">mapNameEN</t>
+  </si>
+  <si>
     <t xml:space="preserve">mapNameDE</t>
   </si>
   <si>
@@ -511,6 +514,9 @@
     <t xml:space="preserve">101</t>
   </si>
   <si>
+    <t xml:space="preserve">Greyfell</t>
+  </si>
+  <si>
     <t xml:space="preserve">Graufurt</t>
   </si>
   <si>
@@ -538,6 +544,9 @@
     <t xml:space="preserve">104</t>
   </si>
   <si>
+    <t xml:space="preserve">Leafshade</t>
+  </si>
+  <si>
     <t xml:space="preserve">Schattenhain</t>
   </si>
   <si>
@@ -547,6 +556,9 @@
     <t xml:space="preserve">105</t>
   </si>
   <si>
+    <t xml:space="preserve">The Shiel</t>
+  </si>
+  <si>
     <t xml:space="preserve">Shiel</t>
   </si>
   <si>
@@ -565,6 +577,9 @@
     <t xml:space="preserve">107</t>
   </si>
   <si>
+    <t xml:space="preserve">Icegate Marsh</t>
+  </si>
+  <si>
     <t xml:space="preserve">Frostmarschen</t>
   </si>
   <si>
@@ -574,6 +589,9 @@
     <t xml:space="preserve">108</t>
   </si>
   <si>
+    <t xml:space="preserve">Northern Windwalls</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nördliche Windwallberge</t>
   </si>
   <si>
@@ -583,6 +601,9 @@
     <t xml:space="preserve">109</t>
   </si>
   <si>
+    <t xml:space="preserve">Southern Windwalls</t>
+  </si>
+  <si>
     <t xml:space="preserve">Südliche Windwallberge</t>
   </si>
   <si>
@@ -592,6 +613,9 @@
     <t xml:space="preserve">110</t>
   </si>
   <si>
+    <t xml:space="preserve">Stoneblade Mountains</t>
+  </si>
+  <si>
     <t xml:space="preserve">Schwertfels</t>
   </si>
   <si>
@@ -601,6 +625,9 @@
     <t xml:space="preserve">111</t>
   </si>
   <si>
+    <t xml:space="preserve">Greydusk Vale</t>
+  </si>
+  <si>
     <t xml:space="preserve">Grauschattental</t>
   </si>
   <si>
@@ -610,6 +637,9 @@
     <t xml:space="preserve">112</t>
   </si>
   <si>
+    <t xml:space="preserve">Howling Mounds</t>
+  </si>
+  <si>
     <t xml:space="preserve">Klagende Steine</t>
   </si>
   <si>
@@ -619,6 +649,9 @@
     <t xml:space="preserve">113</t>
   </si>
   <si>
+    <t xml:space="preserve">Whisper</t>
+  </si>
+  <si>
     <t xml:space="preserve">Wisper</t>
   </si>
   <si>
@@ -628,6 +661,9 @@
     <t xml:space="preserve">114</t>
   </si>
   <si>
+    <t xml:space="preserve">The Godwall</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gottwall</t>
   </si>
   <si>
@@ -646,6 +682,9 @@
     <t xml:space="preserve">116</t>
   </si>
   <si>
+    <t xml:space="preserve">Farlorn’s Hope</t>
+  </si>
+  <si>
     <t xml:space="preserve">Farlorns Heim</t>
   </si>
   <si>
@@ -655,6 +694,9 @@
     <t xml:space="preserve">117</t>
   </si>
   <si>
+    <t xml:space="preserve">The Rift</t>
+  </si>
+  <si>
     <t xml:space="preserve">Spalt</t>
   </si>
   <si>
@@ -664,6 +706,9 @@
     <t xml:space="preserve">118</t>
   </si>
   <si>
+    <t xml:space="preserve">Southern Godmark</t>
+  </si>
+  <si>
     <t xml:space="preserve">Südliche Gottmark</t>
   </si>
   <si>
@@ -673,6 +718,9 @@
     <t xml:space="preserve">119</t>
   </si>
   <si>
+    <t xml:space="preserve">Nightwhisper Dale</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nachtflüstertal</t>
   </si>
   <si>
@@ -682,6 +730,9 @@
     <t xml:space="preserve">120</t>
   </si>
   <si>
+    <t xml:space="preserve">Breathing Forest</t>
+  </si>
+  <si>
     <t xml:space="preserve">Der atmende Wald</t>
   </si>
   <si>
@@ -691,6 +742,9 @@
     <t xml:space="preserve">121</t>
   </si>
   <si>
+    <t xml:space="preserve">Sharrowdale</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sharrow</t>
   </si>
   <si>
@@ -709,6 +763,9 @@
     <t xml:space="preserve">202</t>
   </si>
   <si>
+    <t xml:space="preserve">Stormcleaver Rocks</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sturmfelsen</t>
   </si>
   <si>
@@ -718,6 +775,9 @@
     <t xml:space="preserve">203</t>
   </si>
   <si>
+    <t xml:space="preserve">Echo Swamps</t>
+  </si>
+  <si>
     <t xml:space="preserve">Echosümpfe</t>
   </si>
   <si>
@@ -745,6 +805,9 @@
     <t xml:space="preserve">206</t>
   </si>
   <si>
+    <t xml:space="preserve">Winterdeep</t>
+  </si>
+  <si>
     <t xml:space="preserve">Wintertal</t>
   </si>
   <si>
@@ -763,6 +826,9 @@
     <t xml:space="preserve">208</t>
   </si>
   <si>
+    <t xml:space="preserve">Nevershade Frontier</t>
+  </si>
+  <si>
     <t xml:space="preserve">Schattengrenze</t>
   </si>
   <si>
@@ -781,6 +847,9 @@
     <t xml:space="preserve">210</t>
   </si>
   <si>
+    <t xml:space="preserve">Firefangs</t>
+  </si>
+  <si>
     <t xml:space="preserve">Glutfänge</t>
   </si>
   <si>
@@ -790,6 +859,9 @@
     <t xml:space="preserve">211</t>
   </si>
   <si>
+    <t xml:space="preserve">The Abyss</t>
+  </si>
+  <si>
     <t xml:space="preserve">Der Abgrund</t>
   </si>
   <si>
@@ -799,6 +871,9 @@
     <t xml:space="preserve">212</t>
   </si>
   <si>
+    <t xml:space="preserve">Frostweaver Rift</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gletscherbruch</t>
   </si>
   <si>
@@ -808,6 +883,9 @@
     <t xml:space="preserve">301</t>
   </si>
   <si>
+    <t xml:space="preserve">Blackwater Coast</t>
+  </si>
+  <si>
     <t xml:space="preserve">Schwarze Küste</t>
   </si>
   <si>
@@ -817,6 +895,9 @@
     <t xml:space="preserve">302</t>
   </si>
   <si>
+    <t xml:space="preserve">City of Souls</t>
+  </si>
+  <si>
     <t xml:space="preserve">Stadt der Seelen</t>
   </si>
   <si>
@@ -826,6 +907,9 @@
     <t xml:space="preserve">303</t>
   </si>
   <si>
+    <t xml:space="preserve">Onyx Shores</t>
+  </si>
+  <si>
     <t xml:space="preserve">Onyxbucht</t>
   </si>
   <si>
@@ -844,6 +928,9 @@
     <t xml:space="preserve">305</t>
   </si>
   <si>
+    <t xml:space="preserve">Dryad Cove</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dryadenhain</t>
   </si>
   <si>
@@ -853,6 +940,9 @@
     <t xml:space="preserve">306</t>
   </si>
   <si>
+    <t xml:space="preserve">Red Waste</t>
+  </si>
+  <si>
     <t xml:space="preserve">Rote Wüste</t>
   </si>
   <si>
@@ -862,6 +952,9 @@
     <t xml:space="preserve">307</t>
   </si>
   <si>
+    <t xml:space="preserve">Raven Pass</t>
+  </si>
+  <si>
     <t xml:space="preserve">Rabenpass</t>
   </si>
   <si>
@@ -871,6 +964,9 @@
     <t xml:space="preserve">308</t>
   </si>
   <si>
+    <t xml:space="preserve">Blazing Stones</t>
+  </si>
+  <si>
     <t xml:space="preserve">Brennende Felsen</t>
   </si>
   <si>
@@ -898,6 +994,9 @@
     <t xml:space="preserve">311</t>
   </si>
   <si>
+    <t xml:space="preserve">The Clockwork Crypts</t>
+  </si>
+  <si>
     <t xml:space="preserve">Uhrwerkhallen</t>
   </si>
   <si>
@@ -907,6 +1006,9 @@
     <t xml:space="preserve">312</t>
   </si>
   <si>
+    <t xml:space="preserve">Darkwind Keep</t>
+  </si>
+  <si>
     <t xml:space="preserve">Wachfeste</t>
   </si>
   <si>
@@ -916,6 +1018,9 @@
     <t xml:space="preserve">313</t>
   </si>
   <si>
+    <t xml:space="preserve">The Gorge</t>
+  </si>
+  <si>
     <t xml:space="preserve">Der Schlund</t>
   </si>
   <si>
@@ -923,6 +1028,9 @@
   </si>
   <si>
     <t xml:space="preserve">314</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Bone Temple</t>
   </si>
   <si>
     <t xml:space="preserve">Knochentempel</t>
@@ -4217,16 +4325,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr defaultColWidth="10.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="9.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="8.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="9.43"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4240,10 +4348,10 @@
         <v>151</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>152</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>153</v>
@@ -4251,1057 +4359,1204 @@
       <c r="G1" s="2" t="s">
         <v>154</v>
       </c>
+      <c r="H1" s="2" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="D2" s="1" t="n">
+        <v>158</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="F2" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="G2" s="1" t="n">
         <v>34</v>
       </c>
-      <c r="G2" s="1" t="n">
+      <c r="H2" s="1" t="n">
         <v>104</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="D3" s="1" t="n">
+        <v>161</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="E3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="F3" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="G3" s="1" t="n">
+      <c r="H3" s="1" t="n">
         <v>73</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="D4" s="1" t="n">
+        <v>165</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="1" t="n">
+      <c r="F4" s="1" t="n">
         <v>256</v>
       </c>
-      <c r="G4" s="1" t="n">
+      <c r="H4" s="1" t="n">
         <v>33</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="D5" s="1" t="n">
+        <v>168</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="E5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="F5" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F5" s="1" t="n">
+      <c r="G5" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="G5" s="1" t="n">
+      <c r="H5" s="1" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="D6" s="1" t="n">
+        <v>171</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="E6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="1" t="n">
+      <c r="F6" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F6" s="1" t="n">
+      <c r="G6" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="G6" s="1" t="n">
+      <c r="H6" s="1" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="D7" s="1" t="n">
+        <v>175</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="E7" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="F7" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F7" s="1" t="n">
+      <c r="G7" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="G7" s="1" t="n">
+      <c r="H7" s="1" t="n">
         <v>32</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="D8" s="1" t="n">
+        <v>179</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="E8" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="F8" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="G8" s="1" t="n">
+      <c r="H8" s="1" t="n">
         <v>33</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="D9" s="1" t="n">
+        <v>182</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="E9" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="1" t="n">
+      <c r="F9" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F9" s="1" t="n">
+      <c r="G9" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="G9" s="1" t="n">
+      <c r="H9" s="1" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="D10" s="1" t="n">
+        <v>186</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="E10" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="F10" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="G10" s="1" t="n">
+      <c r="H10" s="1" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="D11" s="1" t="n">
+        <v>190</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="E11" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="1" t="n">
+      <c r="F11" s="1" t="n">
         <v>1024</v>
       </c>
-      <c r="G11" s="1" t="n">
+      <c r="H11" s="1" t="n">
         <v>73</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="D12" s="1" t="n">
+        <v>194</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="E12" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="1" t="n">
+      <c r="F12" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F12" s="1" t="n">
+      <c r="G12" s="1" t="n">
         <v>34</v>
       </c>
-      <c r="G12" s="1" t="n">
+      <c r="H12" s="1" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="D13" s="1" t="n">
+        <v>198</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="E13" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="1" t="n">
+      <c r="F13" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F13" s="1" t="n">
+      <c r="G13" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="G13" s="1" t="n">
+      <c r="H13" s="1" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="D14" s="1" t="n">
+        <v>202</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="E14" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="1" t="n">
+      <c r="F14" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F14" s="1" t="n">
+      <c r="G14" s="1" t="n">
         <v>29</v>
       </c>
-      <c r="G14" s="1" t="n">
+      <c r="H14" s="1" t="n">
         <v>31</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="D15" s="1" t="n">
+        <v>206</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="E15" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="1" t="n">
+      <c r="F15" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="G15" s="1" t="n">
+      <c r="H15" s="1" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>198</v>
+        <v>209</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="D16" s="1" t="n">
+        <v>210</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E16" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="1" t="n">
+      <c r="F16" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="G16" s="1" t="n">
+      <c r="H16" s="1" t="n">
         <v>33</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="D17" s="1" t="n">
+        <v>214</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="E17" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="1" t="n">
+      <c r="F17" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F17" s="1" t="n">
+      <c r="G17" s="1" t="n">
         <v>28</v>
       </c>
-      <c r="G17" s="1" t="n">
+      <c r="H17" s="1" t="n">
         <v>31</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="D18" s="1" t="n">
+        <v>217</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="E18" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="F18" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="G18" s="1" t="n">
+      <c r="H18" s="1" t="n">
         <v>33</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="D19" s="1" t="n">
+        <v>221</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="E19" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="1" t="n">
+      <c r="F19" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F19" s="1" t="n">
+      <c r="G19" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="G19" s="1" t="n">
+      <c r="H19" s="1" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>210</v>
+        <v>224</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="D20" s="1" t="n">
+        <v>225</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="E20" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E20" s="1" t="n">
+      <c r="F20" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F20" s="1" t="n">
+      <c r="G20" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="G20" s="1" t="n">
+      <c r="H20" s="1" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>213</v>
+        <v>228</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="D21" s="1" t="n">
+        <v>229</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="E21" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="1" t="n">
+      <c r="F21" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F21" s="1" t="n">
+      <c r="G21" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="G21" s="1" t="n">
+      <c r="H21" s="1" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>215</v>
+        <v>231</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>216</v>
+        <v>232</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="D22" s="1" t="n">
+        <v>233</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="E22" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E22" s="1" t="n">
+      <c r="F22" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F22" s="1" t="n">
+      <c r="G22" s="1" t="n">
         <v>29</v>
       </c>
-      <c r="G22" s="1" t="n">
+      <c r="H22" s="1" t="n">
         <v>31</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>218</v>
+        <v>235</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>219</v>
+        <v>236</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="D23" s="1" t="n">
+        <v>237</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="E23" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="1" t="n">
+      <c r="F23" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F23" s="1" t="n">
+      <c r="G23" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="G23" s="1" t="n">
+      <c r="H23" s="1" t="n">
         <v>32</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>221</v>
+        <v>239</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>222</v>
+        <v>240</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="D24" s="1" t="n">
+        <v>241</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="E24" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E24" s="1" t="n">
+      <c r="F24" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F24" s="1" t="n">
+      <c r="G24" s="1" t="n">
         <v>136</v>
       </c>
-      <c r="G24" s="1" t="n">
+      <c r="H24" s="1" t="n">
         <v>146</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>224</v>
+        <v>242</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>225</v>
+        <v>243</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="D25" s="1" t="n">
+        <v>244</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="E25" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E25" s="1" t="n">
+      <c r="F25" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="G25" s="1" t="n">
+      <c r="H25" s="1" t="n">
         <v>148</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>227</v>
+        <v>246</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>228</v>
+        <v>247</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="D26" s="1" t="n">
+        <v>248</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="E26" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E26" s="1" t="n">
+      <c r="F26" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="G26" s="1" t="n">
+      <c r="H26" s="1" t="n">
         <v>148</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>230</v>
+        <v>250</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>231</v>
+        <v>251</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="D27" s="1" t="n">
+        <v>252</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="E27" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E27" s="1" t="n">
+      <c r="F27" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="G27" s="1" t="n">
+      <c r="H27" s="1" t="n">
         <v>33</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>233</v>
+        <v>253</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>234</v>
+        <v>254</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="D28" s="1" t="n">
+        <v>255</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="E28" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E28" s="1" t="n">
+      <c r="F28" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F28" s="1" t="n">
+      <c r="G28" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="G28" s="1" t="n">
+      <c r="H28" s="1" t="n">
         <v>147</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>236</v>
+        <v>256</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>237</v>
+        <v>257</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="D29" s="1" t="n">
+        <v>258</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="E29" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E29" s="1" t="n">
+      <c r="F29" s="1" t="n">
         <v>256</v>
       </c>
-      <c r="G29" s="1" t="n">
+      <c r="H29" s="1" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>239</v>
+        <v>260</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>240</v>
+        <v>261</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="D30" s="1" t="n">
+        <v>262</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="E30" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E30" s="1" t="n">
+      <c r="F30" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="G30" s="1" t="n">
+      <c r="H30" s="1" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>242</v>
+        <v>263</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>243</v>
+        <v>264</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="D31" s="1" t="n">
+        <v>265</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="E31" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E31" s="1" t="n">
+      <c r="F31" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="G31" s="1" t="n">
+      <c r="H31" s="1" t="n">
         <v>146</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>245</v>
+        <v>267</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>246</v>
+        <v>268</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="D32" s="1" t="n">
+        <v>269</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="E32" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E32" s="1" t="n">
+      <c r="F32" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F32" s="1" t="n">
+      <c r="G32" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="G32" s="1" t="n">
+      <c r="H32" s="1" t="n">
         <v>31</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>248</v>
+        <v>270</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>249</v>
+        <v>271</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="D33" s="1" t="n">
+        <v>272</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="E33" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E33" s="1" t="n">
+      <c r="F33" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="G33" s="1" t="n">
+      <c r="H33" s="1" t="n">
         <v>138</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>251</v>
+        <v>274</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>252</v>
+        <v>275</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="D34" s="1" t="n">
+        <v>276</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="E34" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E34" s="1" t="n">
+      <c r="F34" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="G34" s="1" t="n">
+      <c r="H34" s="1" t="n">
         <v>73</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>254</v>
+        <v>278</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>255</v>
+        <v>279</v>
       </c>
       <c r="C35" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="E35" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="F35" s="1" t="n">
         <v>256</v>
       </c>
-      <c r="D35" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E35" s="1" t="n">
-        <v>256</v>
-      </c>
-      <c r="F35" s="1" t="n">
+      <c r="G35" s="1" t="n">
         <v>150</v>
       </c>
-      <c r="G35" s="1" t="n">
+      <c r="H35" s="1" t="n">
         <v>147</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>257</v>
+        <v>282</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>258</v>
+        <v>283</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="D36" s="1" t="n">
+        <v>284</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="E36" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E36" s="1" t="n">
+      <c r="F36" s="1" t="n">
         <v>256</v>
       </c>
-      <c r="G36" s="1" t="n">
+      <c r="H36" s="1" t="n">
         <v>237</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>260</v>
+        <v>286</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>261</v>
+        <v>287</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="D37" s="1" t="n">
+        <v>288</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="E37" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E37" s="1" t="n">
+      <c r="F37" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F37" s="1" t="n">
+      <c r="G37" s="1" t="n">
         <v>150</v>
       </c>
-      <c r="G37" s="1" t="n">
+      <c r="H37" s="1" t="n">
         <v>33</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>263</v>
+        <v>290</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>264</v>
+        <v>291</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="D38" s="1" t="n">
+        <v>292</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="E38" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E38" s="1" t="n">
+      <c r="F38" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F38" s="1" t="n">
+      <c r="G38" s="1" t="n">
         <v>136</v>
       </c>
-      <c r="G38" s="1" t="n">
+      <c r="H38" s="1" t="n">
         <v>236</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>266</v>
+        <v>294</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>267</v>
+        <v>295</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="D39" s="1" t="n">
+        <v>296</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="E39" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E39" s="1" t="n">
+      <c r="F39" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F39" s="1" t="n">
+      <c r="G39" s="1" t="n">
         <v>228</v>
       </c>
-      <c r="G39" s="1" t="n">
+      <c r="H39" s="1" t="n">
         <v>238</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>269</v>
+        <v>297</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>270</v>
+        <v>298</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="D40" s="1" t="n">
+        <v>299</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="E40" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E40" s="1" t="n">
+      <c r="F40" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F40" s="1" t="n">
+      <c r="G40" s="1" t="n">
         <v>137</v>
       </c>
-      <c r="G40" s="1" t="n">
+      <c r="H40" s="1" t="n">
         <v>73</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>273</v>
+        <v>302</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="D41" s="1" t="n">
+        <v>303</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="E41" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E41" s="1" t="n">
+      <c r="F41" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F41" s="1" t="n">
+      <c r="G41" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="G41" s="1" t="n">
+      <c r="H41" s="1" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>275</v>
+        <v>305</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>276</v>
+        <v>306</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="D42" s="1" t="n">
+        <v>307</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="E42" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E42" s="1" t="n">
+      <c r="F42" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F42" s="1" t="n">
+      <c r="G42" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="G42" s="1" t="n">
+      <c r="H42" s="1" t="n">
         <v>236</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>278</v>
+        <v>309</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>279</v>
+        <v>310</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="D43" s="1" t="n">
+        <v>311</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="E43" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E43" s="1" t="n">
+      <c r="F43" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F43" s="1" t="n">
+      <c r="G43" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="G43" s="1" t="n">
+      <c r="H43" s="1" t="n">
         <v>237</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>281</v>
+        <v>313</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>282</v>
+        <v>314</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="D44" s="1" t="n">
+        <v>315</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="E44" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E44" s="1" t="n">
+      <c r="F44" s="1" t="n">
         <v>256</v>
       </c>
-      <c r="F44" s="1" t="n">
+      <c r="G44" s="1" t="n">
         <v>228</v>
       </c>
-      <c r="G44" s="1" t="n">
+      <c r="H44" s="1" t="n">
         <v>33</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>284</v>
+        <v>316</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>285</v>
+        <v>317</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="D45" s="1" t="n">
+        <v>318</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="E45" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E45" s="1" t="n">
+      <c r="F45" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F45" s="1" t="n">
+      <c r="G45" s="1" t="n">
         <v>229</v>
       </c>
-      <c r="G45" s="1" t="n">
+      <c r="H45" s="1" t="n">
         <v>238</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>288</v>
+        <v>320</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="D46" s="1" t="n">
+        <v>321</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="E46" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E46" s="1" t="n">
+      <c r="F46" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="G46" s="1" t="n">
+      <c r="H46" s="1" t="n">
         <v>33</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>290</v>
+        <v>323</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>291</v>
+        <v>324</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="D47" s="1" t="n">
+        <v>325</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="E47" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E47" s="1" t="n">
+      <c r="F47" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F47" s="1" t="n">
+      <c r="G47" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="G47" s="1" t="n">
+      <c r="H47" s="1" t="n">
         <v>236</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>293</v>
+        <v>327</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>294</v>
+        <v>328</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="D48" s="1" t="n">
+        <v>329</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="E48" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E48" s="1" t="n">
+      <c r="F48" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="F48" s="1" t="n">
+      <c r="G48" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="G48" s="1" t="n">
+      <c r="H48" s="1" t="n">
         <v>148</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>296</v>
+        <v>331</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>297</v>
+        <v>332</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="D49" s="1" t="n">
+        <v>333</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="E49" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E49" s="1" t="n">
+      <c r="F49" s="1" t="n">
         <v>512</v>
       </c>
-      <c r="G49" s="1" t="n">
+      <c r="H49" s="1" t="n">
         <v>237</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G49">
-    <sortState ref="A2:G49">
+  <autoFilter ref="A1:H49">
+    <sortState ref="A2:H49">
       <sortCondition ref="A2:A49" customList=""/>
     </sortState>
   </autoFilter>
@@ -5337,24 +5592,24 @@
         <v>149</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>299</v>
+        <v>335</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>300</v>
+        <v>336</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>301</v>
+        <v>337</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>281</v>
+        <v>313</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>130</v>
@@ -5374,7 +5629,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>281</v>
+        <v>313</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>130</v>
@@ -5394,7 +5649,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>281</v>
+        <v>313</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>119</v>
@@ -5414,7 +5669,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>257</v>
+        <v>282</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>165</v>
@@ -5434,7 +5689,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>257</v>
+        <v>282</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>86</v>
@@ -5454,7 +5709,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>257</v>
+        <v>282</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>153</v>
@@ -5474,7 +5729,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>257</v>
+        <v>282</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>160</v>
@@ -5494,7 +5749,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>257</v>
+        <v>282</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>167</v>
@@ -5514,7 +5769,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>257</v>
+        <v>282</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>177</v>
@@ -5534,7 +5789,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>257</v>
+        <v>282</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>191</v>
@@ -5554,7 +5809,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>257</v>
+        <v>282</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>217</v>
@@ -5574,7 +5829,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>257</v>
+        <v>282</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>218</v>
@@ -5594,7 +5849,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>260</v>
+        <v>286</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>376</v>
@@ -5614,7 +5869,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>260</v>
+        <v>286</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>4</v>
@@ -5634,7 +5889,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>263</v>
+        <v>290</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>102</v>
@@ -5654,7 +5909,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>263</v>
+        <v>290</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>189</v>
@@ -5674,7 +5929,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>263</v>
+        <v>290</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>279</v>
@@ -5694,7 +5949,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>263</v>
+        <v>290</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>356</v>
@@ -5714,7 +5969,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>263</v>
+        <v>290</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>420</v>
@@ -5734,7 +5989,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>266</v>
+        <v>294</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>175</v>
@@ -5754,7 +6009,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>266</v>
+        <v>294</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>175</v>
@@ -5774,7 +6029,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>266</v>
+        <v>294</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>175</v>
@@ -5794,7 +6049,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>266</v>
+        <v>294</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>175</v>
@@ -5814,7 +6069,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>269</v>
+        <v>297</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>233</v>
@@ -5834,7 +6089,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>269</v>
+        <v>297</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>167</v>
@@ -5854,7 +6109,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>269</v>
+        <v>297</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>129</v>
@@ -5874,7 +6129,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>269</v>
+        <v>297</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>136</v>
@@ -5894,7 +6149,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>269</v>
+        <v>297</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>136</v>
@@ -5914,7 +6169,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>269</v>
+        <v>297</v>
       </c>
       <c r="B30" s="1" t="n">
         <v>227</v>
@@ -5934,7 +6189,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
       <c r="B31" s="1" t="n">
         <v>160</v>
@@ -5954,7 +6209,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
       <c r="B32" s="1" t="n">
         <v>76</v>
@@ -5974,7 +6229,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
       <c r="B33" s="1" t="n">
         <v>86</v>
@@ -5994,7 +6249,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
       <c r="B34" s="1" t="n">
         <v>104</v>
@@ -6014,7 +6269,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
       <c r="B35" s="1" t="n">
         <v>134</v>
@@ -6034,7 +6289,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
       <c r="B36" s="1" t="n">
         <v>305</v>
@@ -6054,7 +6309,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
       <c r="B37" s="1" t="n">
         <v>507</v>
@@ -6074,7 +6329,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>275</v>
+        <v>305</v>
       </c>
       <c r="B38" s="1" t="n">
         <v>374</v>
@@ -6094,7 +6349,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>275</v>
+        <v>305</v>
       </c>
       <c r="B39" s="1" t="n">
         <v>210</v>
@@ -6114,7 +6369,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>275</v>
+        <v>305</v>
       </c>
       <c r="B40" s="1" t="n">
         <v>111</v>
@@ -6134,7 +6389,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>275</v>
+        <v>305</v>
       </c>
       <c r="B41" s="1" t="n">
         <v>118</v>
@@ -6154,7 +6409,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>275</v>
+        <v>305</v>
       </c>
       <c r="B42" s="1" t="n">
         <v>176</v>
@@ -6174,7 +6429,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>275</v>
+        <v>305</v>
       </c>
       <c r="B43" s="1" t="n">
         <v>193</v>
@@ -6194,7 +6449,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>275</v>
+        <v>305</v>
       </c>
       <c r="B44" s="1" t="n">
         <v>250</v>
@@ -6214,7 +6469,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>275</v>
+        <v>305</v>
       </c>
       <c r="B45" s="1" t="n">
         <v>310</v>
@@ -6234,7 +6489,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>275</v>
+        <v>305</v>
       </c>
       <c r="B46" s="1" t="n">
         <v>353</v>
@@ -6254,7 +6509,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>278</v>
+        <v>309</v>
       </c>
       <c r="B47" s="1" t="n">
         <v>169</v>
@@ -6274,7 +6529,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>278</v>
+        <v>309</v>
       </c>
       <c r="B48" s="1" t="n">
         <v>170</v>
@@ -6294,7 +6549,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>278</v>
+        <v>309</v>
       </c>
       <c r="B49" s="1" t="n">
         <v>262</v>
@@ -6314,7 +6569,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>278</v>
+        <v>309</v>
       </c>
       <c r="B50" s="1" t="n">
         <v>31</v>
@@ -6334,7 +6589,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>278</v>
+        <v>309</v>
       </c>
       <c r="B51" s="1" t="n">
         <v>425</v>
@@ -6354,7 +6609,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>278</v>
+        <v>309</v>
       </c>
       <c r="B52" s="1" t="n">
         <v>390</v>
@@ -6374,7 +6629,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>278</v>
+        <v>309</v>
       </c>
       <c r="B53" s="1" t="n">
         <v>353</v>
@@ -6394,7 +6649,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>284</v>
+        <v>316</v>
       </c>
       <c r="B54" s="1" t="n">
         <v>388</v>
@@ -6414,7 +6669,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>284</v>
+        <v>316</v>
       </c>
       <c r="B55" s="1" t="n">
         <v>396</v>
@@ -6434,7 +6689,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>284</v>
+        <v>316</v>
       </c>
       <c r="B56" s="1" t="n">
         <v>49</v>
@@ -6454,7 +6709,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>284</v>
+        <v>316</v>
       </c>
       <c r="B57" s="1" t="n">
         <v>412</v>
@@ -6474,7 +6729,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>284</v>
+        <v>316</v>
       </c>
       <c r="B58" s="1" t="n">
         <v>72</v>
@@ -6494,7 +6749,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>284</v>
+        <v>316</v>
       </c>
       <c r="B59" s="1" t="n">
         <v>190</v>
@@ -6514,7 +6769,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="B60" s="1" t="n">
         <v>139</v>
@@ -6534,7 +6789,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="B61" s="1" t="n">
         <v>223</v>
@@ -6554,7 +6809,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="B62" s="1" t="n">
         <v>310</v>
@@ -6574,7 +6829,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="B63" s="1" t="n">
         <v>138</v>
@@ -6594,7 +6849,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="B64" s="1" t="n">
         <v>223</v>
@@ -6614,7 +6869,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="B65" s="1" t="n">
         <v>313</v>
@@ -6634,7 +6889,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="B66" s="1" t="n">
         <v>310</v>
@@ -6654,7 +6909,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="B67" s="1" t="n">
         <v>225</v>
@@ -6674,7 +6929,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="B68" s="1" t="n">
         <v>138</v>
@@ -6694,7 +6949,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="B69" s="1" t="n">
         <v>438</v>
@@ -6714,7 +6969,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="B70" s="1" t="n">
         <v>433</v>
@@ -6734,7 +6989,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="B71" s="1" t="n">
         <v>426</v>
@@ -6754,7 +7009,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="B72" s="1" t="n">
         <v>426</v>
@@ -6774,7 +7029,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="B73" s="1" t="n">
         <v>437</v>
@@ -6794,7 +7049,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="1" t="s">
-        <v>290</v>
+        <v>323</v>
       </c>
       <c r="B74" s="1" t="n">
         <v>406</v>
@@ -6814,7 +7069,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="1" t="s">
-        <v>290</v>
+        <v>323</v>
       </c>
       <c r="B75" s="1" t="n">
         <v>422</v>
@@ -6834,7 +7089,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="s">
-        <v>290</v>
+        <v>323</v>
       </c>
       <c r="B76" s="1" t="n">
         <v>431</v>
@@ -6854,7 +7109,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="1" t="s">
-        <v>290</v>
+        <v>323</v>
       </c>
       <c r="B77" s="1" t="n">
         <v>180</v>
@@ -6874,7 +7129,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="1" t="s">
-        <v>290</v>
+        <v>323</v>
       </c>
       <c r="B78" s="1" t="n">
         <v>288</v>
@@ -6894,7 +7149,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="1" t="s">
-        <v>290</v>
+        <v>323</v>
       </c>
       <c r="B79" s="1" t="n">
         <v>320</v>
@@ -6914,7 +7169,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="1" t="s">
-        <v>290</v>
+        <v>323</v>
       </c>
       <c r="B80" s="1" t="n">
         <v>354</v>
@@ -6934,7 +7189,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="s">
-        <v>293</v>
+        <v>327</v>
       </c>
       <c r="B81" s="1" t="n">
         <v>257</v>
@@ -6954,7 +7209,7 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="s">
-        <v>293</v>
+        <v>327</v>
       </c>
       <c r="B82" s="1" t="n">
         <v>88</v>
@@ -6974,7 +7229,7 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="s">
-        <v>293</v>
+        <v>327</v>
       </c>
       <c r="B83" s="1" t="n">
         <v>432</v>
@@ -6994,7 +7249,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="1" t="s">
-        <v>293</v>
+        <v>327</v>
       </c>
       <c r="B84" s="1" t="n">
         <v>263</v>
@@ -7014,7 +7269,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="1" t="s">
-        <v>296</v>
+        <v>331</v>
       </c>
       <c r="B85" s="1" t="n">
         <v>444</v>
@@ -7034,7 +7289,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="s">
-        <v>296</v>
+        <v>331</v>
       </c>
       <c r="B86" s="1" t="n">
         <v>430</v>
@@ -7054,7 +7309,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="1" t="s">
-        <v>296</v>
+        <v>331</v>
       </c>
       <c r="B87" s="1" t="n">
         <v>483</v>
@@ -7074,7 +7329,7 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="1" t="s">
-        <v>296</v>
+        <v>331</v>
       </c>
       <c r="B88" s="1" t="n">
         <v>109</v>
@@ -7094,7 +7349,7 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="1" t="s">
-        <v>296</v>
+        <v>331</v>
       </c>
       <c r="B89" s="1" t="n">
         <v>195</v>
@@ -7114,7 +7369,7 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="1" t="s">
-        <v>296</v>
+        <v>331</v>
       </c>
       <c r="B90" s="1" t="n">
         <v>122</v>
@@ -7134,7 +7389,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="1" t="s">
-        <v>221</v>
+        <v>239</v>
       </c>
       <c r="B91" s="1" t="n">
         <v>101</v>
@@ -7154,7 +7409,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="1" t="s">
-        <v>221</v>
+        <v>239</v>
       </c>
       <c r="B92" s="1" t="n">
         <v>271</v>
@@ -7174,7 +7429,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="1" t="s">
-        <v>221</v>
+        <v>239</v>
       </c>
       <c r="B93" s="1" t="n">
         <v>228</v>
@@ -7194,7 +7449,7 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="1" t="s">
-        <v>221</v>
+        <v>239</v>
       </c>
       <c r="B94" s="1" t="n">
         <v>205</v>
@@ -7214,7 +7469,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="1" t="s">
-        <v>224</v>
+        <v>242</v>
       </c>
       <c r="B95" s="1" t="n">
         <v>136</v>
@@ -7234,7 +7489,7 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="1" t="s">
-        <v>224</v>
+        <v>242</v>
       </c>
       <c r="B96" s="1" t="n">
         <v>123</v>
@@ -7254,7 +7509,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="1" t="s">
-        <v>224</v>
+        <v>242</v>
       </c>
       <c r="B97" s="1" t="n">
         <v>300</v>
@@ -7274,7 +7529,7 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="1" t="s">
-        <v>224</v>
+        <v>242</v>
       </c>
       <c r="B98" s="1" t="n">
         <v>318</v>
@@ -7294,7 +7549,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="1" t="s">
-        <v>224</v>
+        <v>242</v>
       </c>
       <c r="B99" s="1" t="n">
         <v>183</v>
@@ -7314,7 +7569,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="1" t="s">
-        <v>224</v>
+        <v>242</v>
       </c>
       <c r="B100" s="1" t="n">
         <v>194</v>
@@ -7334,7 +7589,7 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="1" t="s">
-        <v>227</v>
+        <v>246</v>
       </c>
       <c r="B101" s="1" t="n">
         <v>510</v>
@@ -7354,7 +7609,7 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="1" t="s">
-        <v>227</v>
+        <v>246</v>
       </c>
       <c r="B102" s="1" t="n">
         <v>94</v>
@@ -7374,7 +7629,7 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="1" t="s">
-        <v>230</v>
+        <v>250</v>
       </c>
       <c r="B103" s="1" t="n">
         <v>370</v>
@@ -7394,7 +7649,7 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="1" t="s">
-        <v>230</v>
+        <v>250</v>
       </c>
       <c r="B104" s="1" t="n">
         <v>164</v>
@@ -7414,7 +7669,7 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="1" t="s">
-        <v>230</v>
+        <v>250</v>
       </c>
       <c r="B105" s="1" t="n">
         <v>90</v>
@@ -7434,7 +7689,7 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="1" t="s">
-        <v>230</v>
+        <v>250</v>
       </c>
       <c r="B106" s="1" t="n">
         <v>228</v>
@@ -7454,7 +7709,7 @@
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="1" t="s">
-        <v>230</v>
+        <v>250</v>
       </c>
       <c r="B107" s="1" t="n">
         <v>339</v>
@@ -7474,7 +7729,7 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="1" t="s">
-        <v>230</v>
+        <v>250</v>
       </c>
       <c r="B108" s="1" t="n">
         <v>508</v>
@@ -7494,7 +7749,7 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="1" t="s">
-        <v>233</v>
+        <v>253</v>
       </c>
       <c r="B109" s="1" t="n">
         <v>240</v>
@@ -7514,7 +7769,7 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="1" t="s">
-        <v>233</v>
+        <v>253</v>
       </c>
       <c r="B110" s="1" t="n">
         <v>240</v>
@@ -7534,7 +7789,7 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="1" t="s">
-        <v>233</v>
+        <v>253</v>
       </c>
       <c r="B111" s="1" t="n">
         <v>208</v>
@@ -7554,7 +7809,7 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="1" t="s">
-        <v>233</v>
+        <v>253</v>
       </c>
       <c r="B112" s="1" t="n">
         <v>284</v>
@@ -7574,7 +7829,7 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="1" t="s">
-        <v>233</v>
+        <v>253</v>
       </c>
       <c r="B113" s="1" t="n">
         <v>299</v>
@@ -7594,7 +7849,7 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="1" t="s">
-        <v>239</v>
+        <v>260</v>
       </c>
       <c r="B114" s="1" t="n">
         <v>135</v>
@@ -7614,7 +7869,7 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="1" t="s">
-        <v>239</v>
+        <v>260</v>
       </c>
       <c r="B115" s="1" t="n">
         <v>367</v>
@@ -7634,7 +7889,7 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="1" t="s">
-        <v>242</v>
+        <v>263</v>
       </c>
       <c r="B116" s="1" t="n">
         <v>100</v>
@@ -7654,7 +7909,7 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="1" t="s">
-        <v>242</v>
+        <v>263</v>
       </c>
       <c r="B117" s="1" t="n">
         <v>100</v>
@@ -7674,7 +7929,7 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="1" t="s">
-        <v>242</v>
+        <v>263</v>
       </c>
       <c r="B118" s="1" t="n">
         <v>130</v>
@@ -7694,7 +7949,7 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="1" t="s">
-        <v>242</v>
+        <v>263</v>
       </c>
       <c r="B119" s="1" t="n">
         <v>135</v>
@@ -7714,7 +7969,7 @@
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="1" t="s">
-        <v>245</v>
+        <v>267</v>
       </c>
       <c r="B120" s="1" t="n">
         <v>381</v>
@@ -7734,7 +7989,7 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="1" t="s">
-        <v>245</v>
+        <v>267</v>
       </c>
       <c r="B121" s="1" t="n">
         <v>142</v>
@@ -7754,7 +8009,7 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="1" t="s">
-        <v>245</v>
+        <v>267</v>
       </c>
       <c r="B122" s="1" t="n">
         <v>142</v>
@@ -7774,7 +8029,7 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="1" t="s">
-        <v>248</v>
+        <v>270</v>
       </c>
       <c r="B123" s="1" t="n">
         <v>308</v>
@@ -7794,7 +8049,7 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="1" t="s">
-        <v>248</v>
+        <v>270</v>
       </c>
       <c r="B124" s="1" t="n">
         <v>360</v>
@@ -7814,7 +8069,7 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="1" t="s">
-        <v>248</v>
+        <v>270</v>
       </c>
       <c r="B125" s="1" t="n">
         <v>242</v>
@@ -7834,7 +8089,7 @@
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="1" t="s">
-        <v>251</v>
+        <v>274</v>
       </c>
       <c r="B126" s="1" t="n">
         <v>153</v>
@@ -7854,7 +8109,7 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="1" t="s">
-        <v>251</v>
+        <v>274</v>
       </c>
       <c r="B127" s="1" t="n">
         <v>184</v>
@@ -7874,7 +8129,7 @@
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="1" t="s">
-        <v>251</v>
+        <v>274</v>
       </c>
       <c r="B128" s="1" t="n">
         <v>210</v>
@@ -7894,7 +8149,7 @@
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="1" t="s">
-        <v>251</v>
+        <v>274</v>
       </c>
       <c r="B129" s="1" t="n">
         <v>230</v>
@@ -7914,7 +8169,7 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="1" t="s">
-        <v>251</v>
+        <v>274</v>
       </c>
       <c r="B130" s="1" t="n">
         <v>250</v>
@@ -7934,7 +8189,7 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="1" t="s">
-        <v>251</v>
+        <v>274</v>
       </c>
       <c r="B131" s="1" t="n">
         <v>290</v>
@@ -7954,7 +8209,7 @@
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="1" t="s">
-        <v>251</v>
+        <v>274</v>
       </c>
       <c r="B132" s="1" t="n">
         <v>323</v>
@@ -7974,7 +8229,7 @@
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="1" t="s">
-        <v>251</v>
+        <v>274</v>
       </c>
       <c r="B133" s="1" t="n">
         <v>297</v>
@@ -7994,7 +8249,7 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="1" t="s">
-        <v>251</v>
+        <v>274</v>
       </c>
       <c r="B134" s="1" t="n">
         <v>331</v>
@@ -8014,7 +8269,7 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="1" t="s">
-        <v>251</v>
+        <v>274</v>
       </c>
       <c r="B135" s="1" t="n">
         <v>265</v>
@@ -8034,7 +8289,7 @@
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="1" t="s">
-        <v>251</v>
+        <v>274</v>
       </c>
       <c r="B136" s="1" t="n">
         <v>264</v>
@@ -8054,7 +8309,7 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="1" t="s">
-        <v>254</v>
+        <v>278</v>
       </c>
       <c r="B137" s="1" t="n">
         <v>19</v>
@@ -8074,7 +8329,7 @@
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="1" t="s">
-        <v>254</v>
+        <v>278</v>
       </c>
       <c r="B138" s="1" t="n">
         <v>80</v>
@@ -8094,7 +8349,7 @@
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="1" t="s">
-        <v>254</v>
+        <v>278</v>
       </c>
       <c r="B139" s="1" t="n">
         <v>122</v>
@@ -8114,7 +8369,7 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B140" s="1" t="n">
         <v>425</v>
@@ -8134,7 +8389,7 @@
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B141" s="1" t="n">
         <v>425</v>
@@ -8154,7 +8409,7 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B142" s="1" t="n">
         <v>425</v>
@@ -8174,7 +8429,7 @@
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B143" s="1" t="n">
         <v>425</v>
@@ -8194,7 +8449,7 @@
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B144" s="1" t="n">
         <v>425</v>
@@ -8214,7 +8469,7 @@
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B145" s="1" t="n">
         <v>160</v>
@@ -8234,7 +8489,7 @@
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B146" s="1" t="n">
         <v>146</v>
@@ -8254,7 +8509,7 @@
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B147" s="1" t="n">
         <v>222</v>
@@ -8274,7 +8529,7 @@
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B148" s="1" t="n">
         <v>130</v>
@@ -8294,7 +8549,7 @@
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B149" s="1" t="n">
         <v>252</v>
@@ -8314,7 +8569,7 @@
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B150" s="1" t="n">
         <v>418</v>
@@ -8334,7 +8589,7 @@
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B151" s="1" t="n">
         <v>460</v>
@@ -8354,7 +8609,7 @@
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="1" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B152" s="1" t="n">
         <v>375</v>
@@ -8374,7 +8629,7 @@
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="1" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B153" s="1" t="n">
         <v>510</v>
@@ -8394,7 +8649,7 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="1" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B154" s="1" t="n">
         <v>298</v>
@@ -8414,7 +8669,7 @@
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="1" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B155" s="1" t="n">
         <v>93</v>
@@ -8434,7 +8689,7 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="1" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B156" s="1" t="n">
         <v>80</v>
@@ -8454,7 +8709,7 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="1" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B157" s="1" t="n">
         <v>75</v>
@@ -8474,7 +8729,7 @@
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="1" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B158" s="1" t="n">
         <v>271</v>
@@ -8494,7 +8749,7 @@
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="1" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B159" s="1" t="n">
         <v>299</v>
@@ -8514,7 +8769,7 @@
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="1" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B160" s="1" t="n">
         <v>169</v>
@@ -8534,7 +8789,7 @@
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="1" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B161" s="1" t="n">
         <v>207</v>
@@ -8554,7 +8809,7 @@
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="1" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B162" s="1" t="n">
         <v>145</v>
@@ -8574,7 +8829,7 @@
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="1" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B163" s="1" t="n">
         <v>503</v>
@@ -8594,7 +8849,7 @@
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="1" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B164" s="1" t="n">
         <v>267</v>
@@ -8614,7 +8869,7 @@
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="1" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B165" s="1" t="n">
         <v>425</v>
@@ -8634,7 +8889,7 @@
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="1" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B166" s="1" t="n">
         <v>182</v>
@@ -8654,7 +8909,7 @@
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="1" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B167" s="1" t="n">
         <v>195</v>
@@ -8674,7 +8929,7 @@
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="1" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B168" s="1" t="n">
         <v>322</v>
@@ -8694,7 +8949,7 @@
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="1" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B169" s="1" t="n">
         <v>334</v>
@@ -8714,7 +8969,7 @@
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="1" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B170" s="1" t="n">
         <v>350</v>
@@ -8734,7 +8989,7 @@
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="1" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B171" s="1" t="n">
         <v>368</v>
@@ -8754,7 +9009,7 @@
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="1" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B172" s="1" t="n">
         <v>676</v>
@@ -8774,7 +9029,7 @@
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="1" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="B173" s="1" t="n">
         <v>362</v>
@@ -8794,7 +9049,7 @@
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="1" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="B174" s="1" t="n">
         <v>150</v>
@@ -8814,7 +9069,7 @@
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="1" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B175" s="1" t="n">
         <v>96</v>
@@ -8834,7 +9089,7 @@
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="1" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B176" s="1" t="n">
         <v>139</v>
@@ -8854,7 +9109,7 @@
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="1" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B177" s="1" t="n">
         <v>96</v>
@@ -8874,7 +9129,7 @@
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="1" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B178" s="1" t="n">
         <v>95</v>
@@ -8894,7 +9149,7 @@
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="1" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B179" s="1" t="n">
         <v>219</v>
@@ -8914,7 +9169,7 @@
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="1" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B180" s="1" t="n">
         <v>240</v>
@@ -8934,7 +9189,7 @@
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="1" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B181" s="1" t="n">
         <v>250</v>
@@ -8954,7 +9209,7 @@
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="1" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B182" s="1" t="n">
         <v>260</v>
@@ -8974,7 +9229,7 @@
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="1" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B183" s="1" t="n">
         <v>174</v>
@@ -8994,7 +9249,7 @@
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="1" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="B184" s="1" t="n">
         <v>318</v>
@@ -9014,7 +9269,7 @@
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="1" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="B185" s="1" t="n">
         <v>318</v>
@@ -9034,7 +9289,7 @@
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="1" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="B186" s="1" t="n">
         <v>430</v>
@@ -9054,7 +9309,7 @@
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="1" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="B187" s="1" t="n">
         <v>420</v>
@@ -9074,7 +9329,7 @@
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="1" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="B188" s="1" t="n">
         <v>175</v>
@@ -9094,7 +9349,7 @@
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="1" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="B189" s="1" t="n">
         <v>195</v>
@@ -9114,7 +9369,7 @@
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="1" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="B190" s="1" t="n">
         <v>210</v>
@@ -9134,7 +9389,7 @@
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="1" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="B191" s="1" t="n">
         <v>225</v>
@@ -9154,7 +9409,7 @@
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="1" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="B192" s="1" t="n">
         <v>240</v>
@@ -9174,7 +9429,7 @@
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="1" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="B193" s="1" t="n">
         <v>240</v>
@@ -9194,7 +9449,7 @@
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="1" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="B194" s="1" t="n">
         <v>280</v>
@@ -9214,7 +9469,7 @@
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="1" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="B195" s="1" t="n">
         <v>330</v>
@@ -9234,7 +9489,7 @@
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="1" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="B196" s="1" t="n">
         <v>113</v>
@@ -9254,7 +9509,7 @@
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="1" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="B197" s="1" t="n">
         <v>79</v>
@@ -9274,7 +9529,7 @@
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="1" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="B198" s="1" t="n">
         <v>245</v>
@@ -9294,7 +9549,7 @@
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="1" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="B199" s="1" t="n">
         <v>202</v>
@@ -9314,7 +9569,7 @@
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="1" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="B200" s="1" t="n">
         <v>280</v>
@@ -9334,7 +9589,7 @@
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="1" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="B201" s="1" t="n">
         <v>310</v>
@@ -9354,7 +9609,7 @@
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="1" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="B202" s="1" t="n">
         <v>343</v>
@@ -9374,7 +9629,7 @@
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="1" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="B203" s="1" t="n">
         <v>391</v>
@@ -9394,7 +9649,7 @@
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="1" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="B204" s="1" t="n">
         <v>98</v>
@@ -9414,7 +9669,7 @@
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="1" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="B205" s="1" t="n">
         <v>119</v>
@@ -9434,7 +9689,7 @@
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="1" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="B206" s="1" t="n">
         <v>72</v>
@@ -9454,7 +9709,7 @@
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="1" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="B207" s="1" t="n">
         <v>260</v>
@@ -9474,7 +9729,7 @@
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="1" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="B208" s="1" t="n">
         <v>266</v>
@@ -9494,7 +9749,7 @@
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="1" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="B209" s="1" t="n">
         <v>263</v>
@@ -9514,7 +9769,7 @@
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="1" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="B210" s="1" t="n">
         <v>260</v>
@@ -9534,7 +9789,7 @@
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="1" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="B211" s="1" t="n">
         <v>256</v>
@@ -9554,7 +9809,7 @@
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A212" s="1" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="B212" s="1" t="n">
         <v>250</v>
@@ -9574,7 +9829,7 @@
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="1" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="B213" s="1" t="n">
         <v>380</v>
@@ -9594,7 +9849,7 @@
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="1" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="B214" s="1" t="n">
         <v>384</v>
@@ -9614,7 +9869,7 @@
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="1" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="B215" s="1" t="n">
         <v>396</v>
@@ -9634,7 +9889,7 @@
     </row>
     <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="1" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="B216" s="1" t="n">
         <v>320</v>
@@ -9654,7 +9909,7 @@
     </row>
     <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A217" s="1" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="B217" s="1" t="n">
         <v>250</v>
@@ -9674,7 +9929,7 @@
     </row>
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="1" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="B218" s="1" t="n">
         <v>153</v>
@@ -9694,7 +9949,7 @@
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="1" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="B219" s="1" t="n">
         <v>217</v>
@@ -9714,7 +9969,7 @@
     </row>
     <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="1" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="B220" s="1" t="n">
         <v>130</v>
@@ -9734,7 +9989,7 @@
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="1" t="s">
-        <v>218</v>
+        <v>235</v>
       </c>
       <c r="B221" s="1" t="n">
         <v>155</v>
@@ -9754,7 +10009,7 @@
     </row>
     <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="1" t="s">
-        <v>218</v>
+        <v>235</v>
       </c>
       <c r="B222" s="1" t="n">
         <v>323</v>
@@ -9774,7 +10029,7 @@
     </row>
     <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="1" t="s">
-        <v>218</v>
+        <v>235</v>
       </c>
       <c r="B223" s="1" t="n">
         <v>370</v>
@@ -9794,7 +10049,7 @@
     </row>
     <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="1" t="s">
-        <v>218</v>
+        <v>235</v>
       </c>
       <c r="B224" s="1" t="n">
         <v>403</v>

</xml_diff>